<commit_message>
troca de base de dados - nova base Contratos por regional
</commit_message>
<xml_diff>
--- a/data/Contratos DOPSR1 por Regional.xlsx
+++ b/data/Contratos DOPSR1 por Regional.xlsx
@@ -5,10 +5,10 @@
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Luiza Dias\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Luiza Dias\Downloads\Painel - DER\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE031D53-C849-4BF4-97FA-B7B3921F68E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16B16796-9388-4C96-A3F1-E4731BACA739}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1C8EA352-38C0-4FB9-AC63-E123584F04FB}"/>
   </bookViews>
@@ -602,9 +602,9 @@
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" zeroHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.85546875" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="16.85546875" customWidth="1"/>
     <col min="3" max="3" width="16.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.85546875" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="16.85546875" customWidth="1"/>
     <col min="5" max="5" width="29.140625" customWidth="1"/>
     <col min="6" max="6" width="33.5703125" customWidth="1"/>
     <col min="7" max="16384" width="9.140625" hidden="1"/>
@@ -620,7 +620,7 @@
       <c r="C1" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>59</v>
       </c>
       <c r="E1" s="1" t="s">

</xml_diff>